<commit_message>
Remove company filter from backtest predictions
</commit_message>
<xml_diff>
--- a/backtest_vellam.xlsx
+++ b/backtest_vellam.xlsx
@@ -2859,7 +2859,11 @@
           <t>5443</t>
         </is>
       </c>
-      <c r="M15" s="25" t="inlineStr"/>
+      <c r="M15" s="25" t="inlineStr">
+        <is>
+          <t>N+1 - 8854</t>
+        </is>
+      </c>
       <c r="N15" s="25" t="inlineStr"/>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="18">
@@ -2903,7 +2907,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="M16" s="25" t="inlineStr"/>
+      <c r="M16" s="25" t="inlineStr">
+        <is>
+          <t>N+2 - 9744</t>
+        </is>
+      </c>
       <c r="N16" s="25" t="inlineStr"/>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="18">

</xml_diff>